<commit_message>
feat(v2): upgrade enterprise hub with SVG arrow tour, multi-tab training benchmarking, and robust safe dataframe rendering
</commit_message>
<xml_diff>
--- a/datasets/price_petroleum.xlsx
+++ b/datasets/price_petroleum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03-De tai khoa hoc\Code PetroPrediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1612960F-A032-49F8-9BB0-2A1C812F841D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55845ADC-E6B7-4E45-A0CC-6A8DC5EC5D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7421B51F-E542-4E2D-BF88-A6A71F6B402C}"/>
   </bookViews>
@@ -612,7 +612,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K4659"/>
+  <dimension ref="A1:K4663"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9.4140625" style="1" hidden="1" customWidth="1"/>
@@ -77960,6 +77960,74 @@
         <v>159.29</v>
       </c>
     </row>
+    <row r="4660" spans="4:8">
+      <c r="D4660" s="5">
+        <v>46162</v>
+      </c>
+      <c r="E4660" s="6">
+        <v>137.05000000000001</v>
+      </c>
+      <c r="F4660" s="6">
+        <v>135.16999999999999</v>
+      </c>
+      <c r="G4660" s="6">
+        <v>163.92</v>
+      </c>
+      <c r="H4660" s="6">
+        <v>158.31</v>
+      </c>
+    </row>
+    <row r="4661" spans="4:8">
+      <c r="D4661" s="5">
+        <v>46163</v>
+      </c>
+      <c r="E4661" s="6">
+        <v>130.16</v>
+      </c>
+      <c r="F4661" s="6">
+        <v>129.55000000000001</v>
+      </c>
+      <c r="G4661" s="6">
+        <v>156.75</v>
+      </c>
+      <c r="H4661" s="6">
+        <v>153.97999999999999</v>
+      </c>
+    </row>
+    <row r="4662" spans="4:8">
+      <c r="D4662" s="5">
+        <v>46164</v>
+      </c>
+      <c r="E4662" s="6">
+        <v>127.85</v>
+      </c>
+      <c r="F4662" s="6">
+        <v>127.24</v>
+      </c>
+      <c r="G4662" s="6">
+        <v>153.49</v>
+      </c>
+      <c r="H4662" s="6">
+        <v>150.72</v>
+      </c>
+    </row>
+    <row r="4663" spans="4:8">
+      <c r="D4663" s="5">
+        <v>46167</v>
+      </c>
+      <c r="E4663" s="6">
+        <v>124.81</v>
+      </c>
+      <c r="F4663" s="6">
+        <v>124.25</v>
+      </c>
+      <c r="G4663" s="6">
+        <v>143.32</v>
+      </c>
+      <c r="H4663" s="6">
+        <v>140.55000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <autoFilter ref="A1:H3" xr:uid="{6E8F0AB1-E2D8-4E27-8372-67CC5DA2E1D7}">

</xml_diff>